<commit_message>
Extend conditional formatting to all rows (E3:E1000, F3:F1000, G3:H1000), remove HOW TO UPDATE sheet, and bump sw.js cache to v21
</commit_message>
<xml_diff>
--- a/Aerosol Plant Project Tracker.xlsx
+++ b/Aerosol Plant Project Tracker.xlsx
@@ -1,14 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DASHBOARD" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TRACKER" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HOW TO UPDATE" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet name="DASHBOARD" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="TRACKER" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -2531,7 +2530,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -9543,7 +9542,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
   </mergeCells>
-  <conditionalFormatting sqref="E3:E206">
+  <conditionalFormatting sqref="E3:E1000">
     <cfRule type="expression" priority="7" dxfId="7">
       <formula>$E3="High"</formula>
     </cfRule>
@@ -9554,8 +9553,8 @@
       <formula>$E3="Low"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F4:F27 F140:F168">
-    <cfRule type="dataBar" priority="135">
+  <conditionalFormatting sqref="F3:F1000">
+    <cfRule type="dataBar" priority="1">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="1"/>
@@ -9563,120 +9562,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F13">
-    <cfRule type="dataBar" priority="126">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FF4472C4"/>
-      </dataBar>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F28">
-    <cfRule type="dataBar" priority="47">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FF4472C4"/>
-      </dataBar>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F29">
-    <cfRule type="dataBar" priority="38">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FF4472C4"/>
-      </dataBar>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F30">
-    <cfRule type="dataBar" priority="29">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FF4472C4"/>
-      </dataBar>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F3 F31:F137">
-    <cfRule type="dataBar" priority="56">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FF4472C4"/>
-      </dataBar>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F111">
-    <cfRule type="dataBar" priority="109">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FF4472C4"/>
-      </dataBar>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F112">
-    <cfRule type="dataBar" priority="100">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FF4472C4"/>
-      </dataBar>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F126">
-    <cfRule type="dataBar" priority="58">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FF4472C4"/>
-      </dataBar>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F127:F137 F140:F153">
-    <cfRule type="dataBar" priority="57">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FF4472C4"/>
-      </dataBar>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F138">
-    <cfRule type="dataBar" priority="1">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FF4472C4"/>
-      </dataBar>
-    </cfRule>
-    <cfRule type="dataBar" priority="10">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FF4472C4"/>
-      </dataBar>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F139">
-    <cfRule type="dataBar" priority="11">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FF4472C4"/>
-      </dataBar>
-    </cfRule>
-    <cfRule type="dataBar" priority="20">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FF4472C4"/>
-      </dataBar>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G3:H206">
+  <conditionalFormatting sqref="G3:H1000">
     <cfRule type="expression" priority="2" dxfId="4">
       <formula>$G3="Completed"</formula>
     </cfRule>
@@ -9711,232 +9597,12 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J1" location="DASHBOARD!B1" r:id="rId1"/>
+    <hyperlink ref="J1" location="DASHBOARD!B1" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="B1:F16"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
-  <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="62" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="B1" s="106" t="inlineStr">
-        <is>
-          <t>HOW TO UPDATE — QUICK GUIDE</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="24" customHeight="1">
-      <c r="B2" s="27" t="inlineStr">
-        <is>
-          <t>COLUMN / STEP</t>
-        </is>
-      </c>
-      <c r="C2" s="27" t="inlineStr">
-        <is>
-          <t>INSTRUCTION</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="27.75" customHeight="1">
-      <c r="B3" s="28" t="inlineStr">
-        <is>
-          <t>COLUMN</t>
-        </is>
-      </c>
-      <c r="C3" s="29" t="inlineStr">
-        <is>
-          <t>WHAT TO DO</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Arsalan</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="27.75" customHeight="1">
-      <c r="B4" s="30" t="inlineStr">
-        <is>
-          <t>Machine</t>
-        </is>
-      </c>
-      <c r="C4" s="31" t="inlineStr">
-        <is>
-          <t>Click the cell — a dropdown appears. Pick the machine name.</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Saqib</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="27.75" customHeight="1">
-      <c r="B5" s="28" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="C5" s="29" t="inlineStr">
-        <is>
-          <t>Pick Electrical or Mechanical from the dropdown.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="27.75" customHeight="1">
-      <c r="B6" s="30" t="inlineStr">
-        <is>
-          <t>Task Description</t>
-        </is>
-      </c>
-      <c r="C6" s="31" t="inlineStr">
-        <is>
-          <t>Type the task clearly and briefly.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="27.75" customHeight="1">
-      <c r="B7" s="28" t="inlineStr">
-        <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="C7" s="29" t="inlineStr">
-        <is>
-          <t>High = urgent / blocking.  Medium = important.  Low = when possible.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="27.75" customHeight="1">
-      <c r="B8" s="30" t="inlineStr">
-        <is>
-          <t>Progress</t>
-        </is>
-      </c>
-      <c r="C8" s="31" t="inlineStr">
-        <is>
-          <t>Type a number: 0 = not started,  50 = halfway done,  100 = complete.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="27.75" customHeight="1">
-      <c r="B9" s="28" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C9" s="29" t="inlineStr">
-        <is>
-          <t>Pick from dropdown: Not Started / In Progress / Completed / Blocked / Pending Procurement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="27.75" customHeight="1">
-      <c r="B10" s="30" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="C10" s="31" t="inlineStr">
-        <is>
-          <t>Short notes — vendor, reason for delay, Khalid sb instruction, etc.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="27.75" customHeight="1">
-      <c r="B11" s="28" t="inlineStr">
-        <is>
-          <t>Updated</t>
-        </is>
-      </c>
-      <c r="C11" s="29" t="inlineStr">
-        <is>
-          <t>Type today's date when you update any row.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="27.75" customHeight="1">
-      <c r="B12" s="30" t="inlineStr">
-        <is>
-          <t>Add a new task</t>
-        </is>
-      </c>
-      <c r="C12" s="31" t="inlineStr">
-        <is>
-          <t>Scroll to the bottom. Type in the next empty row. All dropdowns work there too.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="27.75" customHeight="1">
-      <c r="B13" s="28" t="inlineStr">
-        <is>
-          <t>Filter by machine</t>
-        </is>
-      </c>
-      <c r="C13" s="29" t="inlineStr">
-        <is>
-          <t>Click the filter arrow (▼) on the Machine column. Tick only the machine you want.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="27.75" customHeight="1">
-      <c r="B14" s="30" t="inlineStr">
-        <is>
-          <t>Hide completed</t>
-        </is>
-      </c>
-      <c r="C14" s="31" t="inlineStr">
-        <is>
-          <t>Click the filter arrow on Status. Untick Completed. Click OK.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="27.75" customHeight="1">
-      <c r="B15" s="28" t="inlineStr">
-        <is>
-          <t>Dashboard links</t>
-        </is>
-      </c>
-      <c r="C15" s="29" t="inlineStr">
-        <is>
-          <t>On the Dashboard, click any machine name (underlined blue) to jump straight to it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="27.75" customHeight="1">
-      <c r="B16" s="30" t="inlineStr">
-        <is>
-          <t>Back to Dashboard</t>
-        </is>
-      </c>
-      <c r="C16" s="31" t="inlineStr">
-        <is>
-          <t>In the Tracker, click '← Dashboard' in the top-right corner of the sheet.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B1:C1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix Dashboard row 18 Decoration Oven #N/A typo and synchronize Table1 tableRef with autoFilterRef to prevent Excel repair error
</commit_message>
<xml_diff>
--- a/Aerosol Plant Project Tracker.xlsx
+++ b/Aerosol Plant Project Tracker.xlsx
@@ -1542,8 +1542,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A2:J168" headerRowCount="1" totalsRowShown="0" headerRowDxfId="19" headerRowBorderDxfId="18" tableBorderDxfId="17">
-  <autoFilter ref="A2:J168"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A2:J1000" headerRowCount="1" totalsRowShown="0" headerRowDxfId="19" headerRowBorderDxfId="18" tableBorderDxfId="17">
+  <autoFilter ref="A2:J1000"/>
   <tableColumns count="10">
     <tableColumn id="1" name="#" dataDxfId="16"/>
     <tableColumn id="2" name="Machine" dataDxfId="15"/>
@@ -2193,31 +2193,31 @@
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="70">
-        <f>HYPERLINK("#TRACKER!B" &amp; (MATCH("decoration  Oven", TRACKER!$B$4:$B$1002, 0) + 2), "🔥 decoration  Oven")</f>
+        <f>HYPERLINK("#TRACKER!B" &amp; (MATCH("Decoration Oven", TRACKER!$B$4:$B$1002, 0) + 2), "🔥 Decoration Oven")</f>
         <v/>
       </c>
       <c r="C18" s="42">
-        <f>COUNTIFS(TRACKER!$B$4:$B$1002,"decoration  Oven",TRACKER!$C$4:$C$1002,"Electrical",TRACKER!$G$4:$G$1002,"&lt;&gt;Completed")</f>
+        <f>COUNTIFS(TRACKER!$B$4:$B$1002,"Decoration Oven",TRACKER!$C$4:$C$1002,"Electrical",TRACKER!$G$4:$G$1002,"&lt;&gt;Completed")</f>
         <v/>
       </c>
       <c r="D18" s="42">
-        <f>COUNTIFS(TRACKER!$B$4:$B$1002,"decoration  Oven",TRACKER!$C$4:$C$1002,"Mechanical",TRACKER!$G$4:$G$1002,"&lt;&gt;Completed")</f>
+        <f>COUNTIFS(TRACKER!$B$4:$B$1002,"Decoration Oven",TRACKER!$C$4:$C$1002,"Mechanical",TRACKER!$G$4:$G$1002,"&lt;&gt;Completed")</f>
         <v/>
       </c>
       <c r="E18" s="43">
-        <f>COUNTIFS(TRACKER!$B$4:$B$1002,"decoration  Oven",TRACKER!$G$4:$G$1002,"&lt;&gt;Completed")-COUNTIFS(TRACKER!$B$4:$B$1002,"decoration  Oven",TRACKER!$C$4:$C$1002,"Electrical",TRACKER!$G$4:$G$1002,"&lt;&gt;Completed")-COUNTIFS(TRACKER!$B$4:$B$1002,"decoration  Oven",TRACKER!$C$4:$C$1002,"Mechanical",TRACKER!$G$4:$G$1002,"&lt;&gt;Completed")</f>
+        <f>COUNTIFS(TRACKER!$B$4:$B$1002,"Decoration Oven",TRACKER!$G$4:$G$1002,"&lt;&gt;Completed")-COUNTIFS(TRACKER!$B$4:$B$1002,"Decoration Oven",TRACKER!$C$4:$C$1002,"Electrical",TRACKER!$G$4:$G$1002,"&lt;&gt;Completed")-COUNTIFS(TRACKER!$B$4:$B$1002,"Decoration Oven",TRACKER!$C$4:$C$1002,"Mechanical",TRACKER!$G$4:$G$1002,"&lt;&gt;Completed")</f>
         <v/>
       </c>
       <c r="F18" s="44">
-        <f>COUNTIFS(TRACKER!$B$4:$B$1002,"decoration  Oven",TRACKER!$G$4:$G$1002,"&lt;&gt;Completed")</f>
+        <f>COUNTIFS(TRACKER!$B$4:$B$1002,"Decoration Oven",TRACKER!$G$4:$G$1002,"&lt;&gt;Completed")</f>
         <v/>
       </c>
       <c r="G18" s="45">
-        <f>COUNTIFS(TRACKER!$B$4:$B$1002,"decoration  Oven",TRACKER!$G$4:$G$1002,"Completed")</f>
+        <f>COUNTIFS(TRACKER!$B$4:$B$1002,"Decoration Oven",TRACKER!$G$4:$G$1002,"Completed")</f>
         <v/>
       </c>
       <c r="H18" s="66">
-        <f>IFERROR(AVERAGEIF(TRACKER!$B$4:$B$1002,"decoration  Oven",TRACKER!$F$4:$F$1002),0)</f>
+        <f>IFERROR(AVERAGEIF(TRACKER!$B$4:$B$1002,"Decoration Oven",TRACKER!$F$4:$F$1002),0)</f>
         <v/>
       </c>
     </row>
@@ -2253,31 +2253,31 @@
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="B20" s="70">
-        <f>HYPERLINK("#TRACKER!B" &amp; (MATCH("Auto strapping machine", TRACKER!$B$4:$B$1002, 0) + 2), "📦 Auto strapping machine")</f>
+        <f>HYPERLINK("#TRACKER!B" &amp; (MATCH("Auto Strapping Machine", TRACKER!$B$4:$B$1002, 0) + 2), "📦 Auto Strapping Machine")</f>
         <v/>
       </c>
       <c r="C20" s="42">
-        <f>COUNTIFS(TRACKER!$B$4:$B$1002,"Auto strapping machine",TRACKER!$C$4:$C$1002,"Electrical",TRACKER!$G$4:$G$1002,"&lt;&gt;Completed")</f>
+        <f>COUNTIFS(TRACKER!$B$4:$B$1002,"Auto Strapping Machine",TRACKER!$C$4:$C$1002,"Electrical",TRACKER!$G$4:$G$1002,"&lt;&gt;Completed")</f>
         <v/>
       </c>
       <c r="D20" s="42">
-        <f>COUNTIFS(TRACKER!$B$4:$B$1002,"Auto strapping machine",TRACKER!$C$4:$C$1002,"Mechanical",TRACKER!$G$4:$G$1002,"&lt;&gt;Completed")</f>
+        <f>COUNTIFS(TRACKER!$B$4:$B$1002,"Auto Strapping Machine",TRACKER!$C$4:$C$1002,"Mechanical",TRACKER!$G$4:$G$1002,"&lt;&gt;Completed")</f>
         <v/>
       </c>
       <c r="E20" s="43">
-        <f>COUNTIFS(TRACKER!$B$4:$B$1002,"Auto strapping machine",TRACKER!$G$4:$G$1002,"&lt;&gt;Completed")-COUNTIFS(TRACKER!$B$4:$B$1002,"Auto strapping machine",TRACKER!$C$4:$C$1002,"Electrical",TRACKER!$G$4:$G$1002,"&lt;&gt;Completed")-COUNTIFS(TRACKER!$B$4:$B$1002,"Auto strapping machine",TRACKER!$C$4:$C$1002,"Mechanical",TRACKER!$G$4:$G$1002,"&lt;&gt;Completed")</f>
+        <f>COUNTIFS(TRACKER!$B$4:$B$1002,"Auto Strapping Machine",TRACKER!$G$4:$G$1002,"&lt;&gt;Completed")-COUNTIFS(TRACKER!$B$4:$B$1002,"Auto Strapping Machine",TRACKER!$C$4:$C$1002,"Electrical",TRACKER!$G$4:$G$1002,"&lt;&gt;Completed")-COUNTIFS(TRACKER!$B$4:$B$1002,"Auto Strapping Machine",TRACKER!$C$4:$C$1002,"Mechanical",TRACKER!$G$4:$G$1002,"&lt;&gt;Completed")</f>
         <v/>
       </c>
       <c r="F20" s="44">
-        <f>COUNTIFS(TRACKER!$B$4:$B$1002,"Auto strapping machine",TRACKER!$G$4:$G$1002,"&lt;&gt;Completed")</f>
+        <f>COUNTIFS(TRACKER!$B$4:$B$1002,"Auto Strapping Machine",TRACKER!$G$4:$G$1002,"&lt;&gt;Completed")</f>
         <v/>
       </c>
       <c r="G20" s="45">
-        <f>COUNTIFS(TRACKER!$B$4:$B$1002,"Auto strapping machine",TRACKER!$G$4:$G$1002,"Completed")</f>
+        <f>COUNTIFS(TRACKER!$B$4:$B$1002,"Auto Strapping Machine",TRACKER!$G$4:$G$1002,"Completed")</f>
         <v/>
       </c>
       <c r="H20" s="66">
-        <f>IFERROR(AVERAGEIF(TRACKER!$B$4:$B$1002,"Auto strapping machine",TRACKER!$F$4:$F$1002),0)</f>
+        <f>IFERROR(AVERAGEIF(TRACKER!$B$4:$B$1002,"Auto Strapping Machine",TRACKER!$F$4:$F$1002),0)</f>
         <v/>
       </c>
     </row>

</xml_diff>